<commit_message>
Fix Copilot toolkit for Einat 2-hour foundations workshop
Separate foundations entry from AI-leaders tools; rebuild declarative
agent packages; publish skills via .nojekyll and ZIP; reconcile demo
kit accounting; relabel training simulator as rule-based; align
prompt-lab session with late Einat decisions.
</commit_message>
<xml_diff>
--- a/demo-kits/logistics/shipments-sla-2026.xlsx
+++ b/demo-kits/logistics/shipments-sla-2026.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="מעקב_משלוחים_ו_SLA" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מעקב_משלוחים_ו_SLA" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -58,11 +61,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -452,7 +456,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>שם לקוח ואלור</t>
+          <t>שם לקוח טריגר</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -517,21 +521,17 @@
           <t>צפון (חיפה)</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
+      <c r="D2" s="2" t="n">
+        <v>46235</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>46237</v>
       </c>
       <c r="F2" t="n">
         <v>2</v>
       </c>
       <c r="G2">
-        <f>DATEVALUE(E2)-DATEVALUE(D2)</f>
+        <f>E2-D2</f>
         <v/>
       </c>
       <c r="H2">
@@ -568,21 +568,17 @@
           <t>מרכז (תל אביב)</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
+      <c r="D3" s="2" t="n">
+        <v>46236</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>46237</v>
       </c>
       <c r="F3" t="n">
         <v>1</v>
       </c>
       <c r="G3">
-        <f>DATEVALUE(E3)-DATEVALUE(D3)</f>
+        <f>E3-D3</f>
         <v/>
       </c>
       <c r="H3">
@@ -619,21 +615,17 @@
           <t>דרום (באר שבע)</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
+      <c r="D4" s="2" t="n">
+        <v>46237</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>46241</v>
       </c>
       <c r="F4" t="n">
         <v>2</v>
       </c>
       <c r="G4">
-        <f>DATEVALUE(E4)-DATEVALUE(D4)</f>
+        <f>E4-D4</f>
         <v/>
       </c>
       <c r="H4">
@@ -670,21 +662,17 @@
           <t>ירושלים והסביבה</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
+      <c r="D5" s="2" t="n">
+        <v>46239</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>46240</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
       </c>
       <c r="G5">
-        <f>DATEVALUE(E5)-DATEVALUE(D5)</f>
+        <f>E5-D5</f>
         <v/>
       </c>
       <c r="H5">
@@ -721,21 +709,17 @@
           <t>מרכז (פתח תקווה)</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
+      <c r="D6" s="2" t="n">
+        <v>46240</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>46241</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
       </c>
       <c r="G6">
-        <f>DATEVALUE(E6)-DATEVALUE(D6)</f>
+        <f>E6-D6</f>
         <v/>
       </c>
       <c r="H6">
@@ -772,21 +756,17 @@
           <t>צפון (כרמיאל)</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>2026-08-08</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
+      <c r="D7" s="2" t="n">
+        <v>46242</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>46246</v>
       </c>
       <c r="F7" t="n">
         <v>2</v>
       </c>
       <c r="G7">
-        <f>DATEVALUE(E7)-DATEVALUE(D7)</f>
+        <f>E7-D7</f>
         <v/>
       </c>
       <c r="H7">
@@ -823,21 +803,17 @@
           <t>מרכז (הרצליה פיתוח)</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
+      <c r="D8" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>46245</v>
       </c>
       <c r="F8" t="n">
         <v>1</v>
       </c>
       <c r="G8">
-        <f>DATEVALUE(E8)-DATEVALUE(D8)</f>
+        <f>E8-D8</f>
         <v/>
       </c>
       <c r="H8">
@@ -874,21 +850,17 @@
           <t>דרום (אילת)</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2026-08-17</t>
-        </is>
+      <c r="D9" s="2" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>46251</v>
       </c>
       <c r="F9" t="n">
         <v>3</v>
       </c>
       <c r="G9">
-        <f>DATEVALUE(E9)-DATEVALUE(D9)</f>
+        <f>E9-D9</f>
         <v/>
       </c>
       <c r="H9">
@@ -925,21 +897,17 @@
           <t>צפון (נצרת)</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>2026-08-15</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>2026-08-16</t>
-        </is>
+      <c r="D10" s="2" t="n">
+        <v>46249</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>46250</v>
       </c>
       <c r="F10" t="n">
         <v>2</v>
       </c>
       <c r="G10">
-        <f>DATEVALUE(E10)-DATEVALUE(D10)</f>
+        <f>E10-D10</f>
         <v/>
       </c>
       <c r="H10">
@@ -976,21 +944,17 @@
           <t>מרכז (רמת גן)</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
+      <c r="D11" s="2" t="n">
+        <v>46252</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>46253</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
       </c>
       <c r="G11">
-        <f>DATEVALUE(E11)-DATEVALUE(D11)</f>
+        <f>E11-D11</f>
         <v/>
       </c>
       <c r="H11">

</xml_diff>